<commit_message>
Add Kazakh teacher screen and document the language switch
Teacher.html is now built by build_bilingual.py from tools/teacher/ with
the same РУС | ҚАЗ switch. Data arriving from the server in Russian (stage
names, self-assessment marks) is shown in Kazakh on the Kazakh screen
through the same dictionary, so filters keep matching. Abbreviations such
as СОР and ДЗ become БЖБ and ҮТ on Kazakh pages. READMEs describe the two
languages and the Kazakh Excel files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiDAJHuFm4XCVFSPWrS8o1
</commit_message>
<xml_diff>
--- a/lessons-8-stats/Кілт_статистика.xlsx
+++ b/lessons-8-stats/Кілт_статистика.xlsx
@@ -525,22 +525,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>СОР 1</t>
+          <t>БЖБ 1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>СОР 2</t>
+          <t>БЖБ 2</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>СОР 3</t>
+          <t>БЖБ 3</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>СОЧ</t>
+          <t>ТЖБ</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>